<commit_message>
Actualizacao das bases e graficos
</commit_message>
<xml_diff>
--- a/Beneficiarios_Indiretos.xlsx
+++ b/Beneficiarios_Indiretos.xlsx
@@ -1363,13 +1363,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DC8ACA8-F79F-45EC-8FED-39D35A70DDC9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAE7EAE8-FE6C-4EF6-839C-D1E5D4294098}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E0DC18F-B25C-47E4-BC11-3B2EA7664FD9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1F66641-2CA7-4374-9621-2C61A63344C9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EADFBA9D-EF02-4A93-AC34-D7D097892274}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02F681C4-2540-4FAD-9F19-A73CB1291F22}"/>
 </file>
</xml_diff>